<commit_message>
data(light-cones): G01-P7-L01 import light cone partition 01
</commit_message>
<xml_diff>
--- a/config/data/ModifierDefinition.xlsx
+++ b/config/data/ModifierDefinition.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R893"/>
+  <dimension ref="A1:R973"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49594,6 +49594,4646 @@
         </is>
       </c>
     </row>
+    <row r="894">
+      <c r="B894" t="n">
+        <v>211001</v>
+      </c>
+      <c r="C894" t="n">
+        <v>210001</v>
+      </c>
+      <c r="E894" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F894" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G894" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H894" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I894" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J894" t="n">
+        <v>213001</v>
+      </c>
+      <c r="K894" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L894" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M894" t="n">
+        <v>0</v>
+      </c>
+      <c r="P894" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q894" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R894" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="B895" t="n">
+        <v>211002</v>
+      </c>
+      <c r="C895" t="n">
+        <v>210001</v>
+      </c>
+      <c r="E895" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F895" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G895" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H895" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I895" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J895" t="n">
+        <v>213002</v>
+      </c>
+      <c r="K895" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L895" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M895" t="n">
+        <v>0</v>
+      </c>
+      <c r="P895" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q895" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R895" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="B896" t="n">
+        <v>211003</v>
+      </c>
+      <c r="C896" t="n">
+        <v>210001</v>
+      </c>
+      <c r="E896" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F896" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G896" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H896" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I896" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J896" t="n">
+        <v>213003</v>
+      </c>
+      <c r="K896" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L896" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M896" t="n">
+        <v>0</v>
+      </c>
+      <c r="P896" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q896" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R896" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="B897" t="n">
+        <v>211004</v>
+      </c>
+      <c r="C897" t="n">
+        <v>210001</v>
+      </c>
+      <c r="E897" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F897" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G897" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H897" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I897" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J897" t="n">
+        <v>213004</v>
+      </c>
+      <c r="K897" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L897" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M897" t="n">
+        <v>0</v>
+      </c>
+      <c r="P897" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q897" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R897" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="B898" t="n">
+        <v>211005</v>
+      </c>
+      <c r="C898" t="n">
+        <v>210001</v>
+      </c>
+      <c r="E898" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F898" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G898" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H898" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I898" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J898" t="n">
+        <v>213005</v>
+      </c>
+      <c r="K898" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L898" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M898" t="n">
+        <v>0</v>
+      </c>
+      <c r="P898" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q898" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R898" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="B899" t="n">
+        <v>211006</v>
+      </c>
+      <c r="C899" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E899" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F899" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G899" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H899" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I899" t="inlineStr">
+        <is>
+          <t>OrdinaryDamage</t>
+        </is>
+      </c>
+      <c r="J899" t="n">
+        <v>213006</v>
+      </c>
+      <c r="K899" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L899" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M899" t="n">
+        <v>0</v>
+      </c>
+      <c r="P899" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q899" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R899" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="B900" t="n">
+        <v>211007</v>
+      </c>
+      <c r="C900" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E900" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F900" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G900" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H900" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I900" t="inlineStr">
+        <is>
+          <t>Dot</t>
+        </is>
+      </c>
+      <c r="J900" t="n">
+        <v>213007</v>
+      </c>
+      <c r="K900" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L900" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M900" t="n">
+        <v>0</v>
+      </c>
+      <c r="P900" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q900" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R900" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="B901" t="n">
+        <v>211008</v>
+      </c>
+      <c r="C901" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E901" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F901" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G901" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H901" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I901" t="inlineStr">
+        <is>
+          <t>AdditionalDamage</t>
+        </is>
+      </c>
+      <c r="J901" t="n">
+        <v>213008</v>
+      </c>
+      <c r="K901" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L901" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M901" t="n">
+        <v>0</v>
+      </c>
+      <c r="P901" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q901" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R901" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="B902" t="n">
+        <v>211009</v>
+      </c>
+      <c r="C902" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E902" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F902" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G902" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H902" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I902" t="inlineStr">
+        <is>
+          <t>JointDamage</t>
+        </is>
+      </c>
+      <c r="J902" t="n">
+        <v>213009</v>
+      </c>
+      <c r="K902" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L902" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M902" t="n">
+        <v>0</v>
+      </c>
+      <c r="P902" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q902" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R902" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="B903" t="n">
+        <v>211010</v>
+      </c>
+      <c r="C903" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E903" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F903" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G903" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H903" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I903" t="inlineStr">
+        <is>
+          <t>ElationDamage</t>
+        </is>
+      </c>
+      <c r="J903" t="n">
+        <v>213010</v>
+      </c>
+      <c r="K903" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L903" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M903" t="n">
+        <v>0</v>
+      </c>
+      <c r="P903" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q903" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R903" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="B904" t="n">
+        <v>211011</v>
+      </c>
+      <c r="C904" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E904" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F904" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G904" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H904" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I904" t="inlineStr">
+        <is>
+          <t>OrdinaryDamage</t>
+        </is>
+      </c>
+      <c r="J904" t="n">
+        <v>213011</v>
+      </c>
+      <c r="K904" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L904" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M904" t="n">
+        <v>0</v>
+      </c>
+      <c r="P904" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q904" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R904" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="B905" t="n">
+        <v>211012</v>
+      </c>
+      <c r="C905" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E905" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F905" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G905" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H905" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I905" t="inlineStr">
+        <is>
+          <t>Dot</t>
+        </is>
+      </c>
+      <c r="J905" t="n">
+        <v>213012</v>
+      </c>
+      <c r="K905" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L905" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M905" t="n">
+        <v>0</v>
+      </c>
+      <c r="P905" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q905" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R905" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="B906" t="n">
+        <v>211013</v>
+      </c>
+      <c r="C906" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E906" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F906" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G906" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H906" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I906" t="inlineStr">
+        <is>
+          <t>AdditionalDamage</t>
+        </is>
+      </c>
+      <c r="J906" t="n">
+        <v>213013</v>
+      </c>
+      <c r="K906" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L906" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M906" t="n">
+        <v>0</v>
+      </c>
+      <c r="P906" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q906" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R906" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="B907" t="n">
+        <v>211014</v>
+      </c>
+      <c r="C907" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E907" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F907" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G907" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H907" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I907" t="inlineStr">
+        <is>
+          <t>JointDamage</t>
+        </is>
+      </c>
+      <c r="J907" t="n">
+        <v>213014</v>
+      </c>
+      <c r="K907" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L907" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M907" t="n">
+        <v>0</v>
+      </c>
+      <c r="P907" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q907" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R907" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="B908" t="n">
+        <v>211015</v>
+      </c>
+      <c r="C908" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E908" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F908" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G908" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H908" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I908" t="inlineStr">
+        <is>
+          <t>ElationDamage</t>
+        </is>
+      </c>
+      <c r="J908" t="n">
+        <v>213015</v>
+      </c>
+      <c r="K908" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L908" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M908" t="n">
+        <v>0</v>
+      </c>
+      <c r="P908" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q908" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R908" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="B909" t="n">
+        <v>211016</v>
+      </c>
+      <c r="C909" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E909" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F909" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G909" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H909" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I909" t="inlineStr">
+        <is>
+          <t>OrdinaryDamage</t>
+        </is>
+      </c>
+      <c r="J909" t="n">
+        <v>213016</v>
+      </c>
+      <c r="K909" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L909" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M909" t="n">
+        <v>0</v>
+      </c>
+      <c r="P909" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q909" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R909" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="B910" t="n">
+        <v>211017</v>
+      </c>
+      <c r="C910" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E910" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F910" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G910" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H910" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I910" t="inlineStr">
+        <is>
+          <t>Dot</t>
+        </is>
+      </c>
+      <c r="J910" t="n">
+        <v>213017</v>
+      </c>
+      <c r="K910" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L910" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M910" t="n">
+        <v>0</v>
+      </c>
+      <c r="P910" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q910" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R910" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="B911" t="n">
+        <v>211018</v>
+      </c>
+      <c r="C911" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E911" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F911" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G911" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H911" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I911" t="inlineStr">
+        <is>
+          <t>AdditionalDamage</t>
+        </is>
+      </c>
+      <c r="J911" t="n">
+        <v>213018</v>
+      </c>
+      <c r="K911" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L911" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M911" t="n">
+        <v>0</v>
+      </c>
+      <c r="P911" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q911" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R911" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="B912" t="n">
+        <v>211019</v>
+      </c>
+      <c r="C912" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E912" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F912" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G912" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H912" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I912" t="inlineStr">
+        <is>
+          <t>JointDamage</t>
+        </is>
+      </c>
+      <c r="J912" t="n">
+        <v>213019</v>
+      </c>
+      <c r="K912" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L912" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M912" t="n">
+        <v>0</v>
+      </c>
+      <c r="P912" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q912" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R912" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="B913" t="n">
+        <v>211020</v>
+      </c>
+      <c r="C913" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E913" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F913" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G913" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H913" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I913" t="inlineStr">
+        <is>
+          <t>ElationDamage</t>
+        </is>
+      </c>
+      <c r="J913" t="n">
+        <v>213020</v>
+      </c>
+      <c r="K913" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L913" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M913" t="n">
+        <v>0</v>
+      </c>
+      <c r="P913" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q913" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R913" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="B914" t="n">
+        <v>211021</v>
+      </c>
+      <c r="C914" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E914" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F914" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G914" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H914" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I914" t="inlineStr">
+        <is>
+          <t>OrdinaryDamage</t>
+        </is>
+      </c>
+      <c r="J914" t="n">
+        <v>213021</v>
+      </c>
+      <c r="K914" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L914" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M914" t="n">
+        <v>0</v>
+      </c>
+      <c r="P914" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q914" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R914" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="B915" t="n">
+        <v>211022</v>
+      </c>
+      <c r="C915" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E915" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F915" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G915" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H915" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I915" t="inlineStr">
+        <is>
+          <t>Dot</t>
+        </is>
+      </c>
+      <c r="J915" t="n">
+        <v>213022</v>
+      </c>
+      <c r="K915" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L915" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M915" t="n">
+        <v>0</v>
+      </c>
+      <c r="P915" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q915" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R915" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="B916" t="n">
+        <v>211023</v>
+      </c>
+      <c r="C916" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E916" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F916" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G916" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H916" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I916" t="inlineStr">
+        <is>
+          <t>AdditionalDamage</t>
+        </is>
+      </c>
+      <c r="J916" t="n">
+        <v>213023</v>
+      </c>
+      <c r="K916" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L916" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M916" t="n">
+        <v>0</v>
+      </c>
+      <c r="P916" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q916" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R916" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="B917" t="n">
+        <v>211024</v>
+      </c>
+      <c r="C917" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E917" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F917" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G917" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H917" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I917" t="inlineStr">
+        <is>
+          <t>JointDamage</t>
+        </is>
+      </c>
+      <c r="J917" t="n">
+        <v>213024</v>
+      </c>
+      <c r="K917" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L917" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M917" t="n">
+        <v>0</v>
+      </c>
+      <c r="P917" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q917" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R917" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="B918" t="n">
+        <v>211025</v>
+      </c>
+      <c r="C918" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E918" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F918" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G918" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H918" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I918" t="inlineStr">
+        <is>
+          <t>ElationDamage</t>
+        </is>
+      </c>
+      <c r="J918" t="n">
+        <v>213025</v>
+      </c>
+      <c r="K918" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L918" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M918" t="n">
+        <v>0</v>
+      </c>
+      <c r="P918" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q918" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R918" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="B919" t="n">
+        <v>211026</v>
+      </c>
+      <c r="C919" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E919" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F919" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G919" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H919" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I919" t="inlineStr">
+        <is>
+          <t>OrdinaryDamage</t>
+        </is>
+      </c>
+      <c r="J919" t="n">
+        <v>213026</v>
+      </c>
+      <c r="K919" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L919" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M919" t="n">
+        <v>0</v>
+      </c>
+      <c r="P919" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q919" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R919" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="B920" t="n">
+        <v>211027</v>
+      </c>
+      <c r="C920" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E920" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F920" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G920" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H920" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I920" t="inlineStr">
+        <is>
+          <t>Dot</t>
+        </is>
+      </c>
+      <c r="J920" t="n">
+        <v>213027</v>
+      </c>
+      <c r="K920" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L920" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M920" t="n">
+        <v>0</v>
+      </c>
+      <c r="P920" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q920" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R920" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="B921" t="n">
+        <v>211028</v>
+      </c>
+      <c r="C921" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E921" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F921" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G921" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H921" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I921" t="inlineStr">
+        <is>
+          <t>AdditionalDamage</t>
+        </is>
+      </c>
+      <c r="J921" t="n">
+        <v>213028</v>
+      </c>
+      <c r="K921" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L921" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M921" t="n">
+        <v>0</v>
+      </c>
+      <c r="P921" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q921" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R921" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="B922" t="n">
+        <v>211029</v>
+      </c>
+      <c r="C922" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E922" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F922" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G922" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H922" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I922" t="inlineStr">
+        <is>
+          <t>JointDamage</t>
+        </is>
+      </c>
+      <c r="J922" t="n">
+        <v>213029</v>
+      </c>
+      <c r="K922" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L922" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M922" t="n">
+        <v>0</v>
+      </c>
+      <c r="P922" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q922" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R922" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="B923" t="n">
+        <v>211030</v>
+      </c>
+      <c r="C923" t="n">
+        <v>210003</v>
+      </c>
+      <c r="E923" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F923" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G923" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="H923" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="I923" t="inlineStr">
+        <is>
+          <t>ElationDamage</t>
+        </is>
+      </c>
+      <c r="J923" t="n">
+        <v>213030</v>
+      </c>
+      <c r="K923" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L923" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M923" t="n">
+        <v>0</v>
+      </c>
+      <c r="P923" t="inlineStr">
+        <is>
+          <t>DamageBoost</t>
+        </is>
+      </c>
+      <c r="Q923" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R923" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="B924" t="n">
+        <v>211031</v>
+      </c>
+      <c r="C924" t="n">
+        <v>210005</v>
+      </c>
+      <c r="E924" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F924" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G924" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H924" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I924" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J924" t="n">
+        <v>213031</v>
+      </c>
+      <c r="K924" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L924" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M924" t="n">
+        <v>0</v>
+      </c>
+      <c r="P924" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q924" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R924" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="B925" t="n">
+        <v>211032</v>
+      </c>
+      <c r="C925" t="n">
+        <v>210005</v>
+      </c>
+      <c r="E925" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F925" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G925" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H925" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I925" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J925" t="n">
+        <v>213032</v>
+      </c>
+      <c r="K925" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L925" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M925" t="n">
+        <v>0</v>
+      </c>
+      <c r="P925" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q925" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R925" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="B926" t="n">
+        <v>211033</v>
+      </c>
+      <c r="C926" t="n">
+        <v>210005</v>
+      </c>
+      <c r="E926" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F926" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G926" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H926" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I926" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J926" t="n">
+        <v>213033</v>
+      </c>
+      <c r="K926" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L926" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M926" t="n">
+        <v>0</v>
+      </c>
+      <c r="P926" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q926" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R926" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="B927" t="n">
+        <v>211034</v>
+      </c>
+      <c r="C927" t="n">
+        <v>210005</v>
+      </c>
+      <c r="E927" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F927" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G927" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H927" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I927" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J927" t="n">
+        <v>213034</v>
+      </c>
+      <c r="K927" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L927" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M927" t="n">
+        <v>0</v>
+      </c>
+      <c r="P927" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q927" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R927" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="B928" t="n">
+        <v>211035</v>
+      </c>
+      <c r="C928" t="n">
+        <v>210005</v>
+      </c>
+      <c r="E928" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F928" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G928" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H928" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I928" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J928" t="n">
+        <v>213035</v>
+      </c>
+      <c r="K928" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L928" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M928" t="n">
+        <v>0</v>
+      </c>
+      <c r="P928" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q928" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R928" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="B929" t="n">
+        <v>211036</v>
+      </c>
+      <c r="C929" t="n">
+        <v>210006</v>
+      </c>
+      <c r="E929" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F929" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G929" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H929" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I929" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J929" t="n">
+        <v>213036</v>
+      </c>
+      <c r="K929" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L929" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M929" t="n">
+        <v>0</v>
+      </c>
+      <c r="P929" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q929" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R929" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="B930" t="n">
+        <v>211037</v>
+      </c>
+      <c r="C930" t="n">
+        <v>210006</v>
+      </c>
+      <c r="E930" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F930" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G930" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H930" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I930" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J930" t="n">
+        <v>213037</v>
+      </c>
+      <c r="K930" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L930" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M930" t="n">
+        <v>0</v>
+      </c>
+      <c r="P930" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q930" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R930" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="B931" t="n">
+        <v>211038</v>
+      </c>
+      <c r="C931" t="n">
+        <v>210006</v>
+      </c>
+      <c r="E931" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F931" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G931" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H931" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I931" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J931" t="n">
+        <v>213038</v>
+      </c>
+      <c r="K931" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L931" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M931" t="n">
+        <v>0</v>
+      </c>
+      <c r="P931" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q931" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R931" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="B932" t="n">
+        <v>211039</v>
+      </c>
+      <c r="C932" t="n">
+        <v>210006</v>
+      </c>
+      <c r="E932" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F932" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G932" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H932" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I932" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J932" t="n">
+        <v>213039</v>
+      </c>
+      <c r="K932" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L932" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M932" t="n">
+        <v>0</v>
+      </c>
+      <c r="P932" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q932" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R932" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="B933" t="n">
+        <v>211040</v>
+      </c>
+      <c r="C933" t="n">
+        <v>210006</v>
+      </c>
+      <c r="E933" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F933" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G933" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H933" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I933" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J933" t="n">
+        <v>213040</v>
+      </c>
+      <c r="K933" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L933" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M933" t="n">
+        <v>0</v>
+      </c>
+      <c r="P933" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q933" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R933" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="B934" t="n">
+        <v>211041</v>
+      </c>
+      <c r="C934" t="n">
+        <v>210008</v>
+      </c>
+      <c r="E934" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F934" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G934" t="inlineStr">
+        <is>
+          <t>BreakEffect</t>
+        </is>
+      </c>
+      <c r="H934" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I934" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J934" t="n">
+        <v>213041</v>
+      </c>
+      <c r="K934" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L934" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M934" t="n">
+        <v>0</v>
+      </c>
+      <c r="P934" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q934" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R934" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="B935" t="n">
+        <v>211042</v>
+      </c>
+      <c r="C935" t="n">
+        <v>210008</v>
+      </c>
+      <c r="E935" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F935" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G935" t="inlineStr">
+        <is>
+          <t>BreakEffect</t>
+        </is>
+      </c>
+      <c r="H935" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I935" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J935" t="n">
+        <v>213042</v>
+      </c>
+      <c r="K935" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L935" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M935" t="n">
+        <v>0</v>
+      </c>
+      <c r="P935" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q935" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R935" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="B936" t="n">
+        <v>211043</v>
+      </c>
+      <c r="C936" t="n">
+        <v>210008</v>
+      </c>
+      <c r="E936" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F936" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G936" t="inlineStr">
+        <is>
+          <t>BreakEffect</t>
+        </is>
+      </c>
+      <c r="H936" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I936" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J936" t="n">
+        <v>213043</v>
+      </c>
+      <c r="K936" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L936" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M936" t="n">
+        <v>0</v>
+      </c>
+      <c r="P936" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q936" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R936" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="B937" t="n">
+        <v>211044</v>
+      </c>
+      <c r="C937" t="n">
+        <v>210008</v>
+      </c>
+      <c r="E937" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F937" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G937" t="inlineStr">
+        <is>
+          <t>BreakEffect</t>
+        </is>
+      </c>
+      <c r="H937" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I937" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J937" t="n">
+        <v>213044</v>
+      </c>
+      <c r="K937" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L937" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M937" t="n">
+        <v>0</v>
+      </c>
+      <c r="P937" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q937" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R937" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="B938" t="n">
+        <v>211045</v>
+      </c>
+      <c r="C938" t="n">
+        <v>210008</v>
+      </c>
+      <c r="E938" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F938" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G938" t="inlineStr">
+        <is>
+          <t>BreakEffect</t>
+        </is>
+      </c>
+      <c r="H938" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I938" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J938" t="n">
+        <v>213045</v>
+      </c>
+      <c r="K938" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L938" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M938" t="n">
+        <v>0</v>
+      </c>
+      <c r="P938" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q938" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R938" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="B939" t="n">
+        <v>211046</v>
+      </c>
+      <c r="C939" t="n">
+        <v>210009</v>
+      </c>
+      <c r="E939" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F939" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G939" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H939" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I939" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J939" t="n">
+        <v>213046</v>
+      </c>
+      <c r="K939" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L939" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M939" t="n">
+        <v>0</v>
+      </c>
+      <c r="P939" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q939" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R939" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="B940" t="n">
+        <v>211047</v>
+      </c>
+      <c r="C940" t="n">
+        <v>210009</v>
+      </c>
+      <c r="E940" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F940" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G940" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H940" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I940" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J940" t="n">
+        <v>213047</v>
+      </c>
+      <c r="K940" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L940" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M940" t="n">
+        <v>0</v>
+      </c>
+      <c r="P940" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q940" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R940" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="B941" t="n">
+        <v>211048</v>
+      </c>
+      <c r="C941" t="n">
+        <v>210009</v>
+      </c>
+      <c r="E941" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F941" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G941" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H941" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I941" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J941" t="n">
+        <v>213048</v>
+      </c>
+      <c r="K941" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L941" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M941" t="n">
+        <v>0</v>
+      </c>
+      <c r="P941" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q941" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R941" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="B942" t="n">
+        <v>211049</v>
+      </c>
+      <c r="C942" t="n">
+        <v>210009</v>
+      </c>
+      <c r="E942" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F942" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G942" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H942" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I942" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J942" t="n">
+        <v>213049</v>
+      </c>
+      <c r="K942" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L942" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M942" t="n">
+        <v>0</v>
+      </c>
+      <c r="P942" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q942" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R942" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="B943" t="n">
+        <v>211050</v>
+      </c>
+      <c r="C943" t="n">
+        <v>210009</v>
+      </c>
+      <c r="E943" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F943" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G943" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H943" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I943" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J943" t="n">
+        <v>213050</v>
+      </c>
+      <c r="K943" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L943" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M943" t="n">
+        <v>0</v>
+      </c>
+      <c r="P943" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q943" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R943" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="B944" t="n">
+        <v>211051</v>
+      </c>
+      <c r="C944" t="n">
+        <v>210010</v>
+      </c>
+      <c r="E944" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F944" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G944" t="inlineStr">
+        <is>
+          <t>Def</t>
+        </is>
+      </c>
+      <c r="H944" t="inlineStr">
+        <is>
+          <t>PercentOfBase</t>
+        </is>
+      </c>
+      <c r="I944" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J944" t="n">
+        <v>213051</v>
+      </c>
+      <c r="K944" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L944" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M944" t="n">
+        <v>0</v>
+      </c>
+      <c r="P944" t="inlineStr">
+        <is>
+          <t>PercentOfBase</t>
+        </is>
+      </c>
+      <c r="Q944" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R944" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="B945" t="n">
+        <v>211052</v>
+      </c>
+      <c r="C945" t="n">
+        <v>210010</v>
+      </c>
+      <c r="E945" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F945" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G945" t="inlineStr">
+        <is>
+          <t>Def</t>
+        </is>
+      </c>
+      <c r="H945" t="inlineStr">
+        <is>
+          <t>PercentOfBase</t>
+        </is>
+      </c>
+      <c r="I945" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J945" t="n">
+        <v>213052</v>
+      </c>
+      <c r="K945" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L945" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M945" t="n">
+        <v>0</v>
+      </c>
+      <c r="P945" t="inlineStr">
+        <is>
+          <t>PercentOfBase</t>
+        </is>
+      </c>
+      <c r="Q945" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R945" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="B946" t="n">
+        <v>211053</v>
+      </c>
+      <c r="C946" t="n">
+        <v>210010</v>
+      </c>
+      <c r="E946" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F946" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G946" t="inlineStr">
+        <is>
+          <t>Def</t>
+        </is>
+      </c>
+      <c r="H946" t="inlineStr">
+        <is>
+          <t>PercentOfBase</t>
+        </is>
+      </c>
+      <c r="I946" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J946" t="n">
+        <v>213053</v>
+      </c>
+      <c r="K946" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L946" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M946" t="n">
+        <v>0</v>
+      </c>
+      <c r="P946" t="inlineStr">
+        <is>
+          <t>PercentOfBase</t>
+        </is>
+      </c>
+      <c r="Q946" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R946" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="B947" t="n">
+        <v>211054</v>
+      </c>
+      <c r="C947" t="n">
+        <v>210010</v>
+      </c>
+      <c r="E947" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F947" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G947" t="inlineStr">
+        <is>
+          <t>Def</t>
+        </is>
+      </c>
+      <c r="H947" t="inlineStr">
+        <is>
+          <t>PercentOfBase</t>
+        </is>
+      </c>
+      <c r="I947" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J947" t="n">
+        <v>213054</v>
+      </c>
+      <c r="K947" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L947" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M947" t="n">
+        <v>0</v>
+      </c>
+      <c r="P947" t="inlineStr">
+        <is>
+          <t>PercentOfBase</t>
+        </is>
+      </c>
+      <c r="Q947" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R947" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="B948" t="n">
+        <v>211055</v>
+      </c>
+      <c r="C948" t="n">
+        <v>210010</v>
+      </c>
+      <c r="E948" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F948" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G948" t="inlineStr">
+        <is>
+          <t>Def</t>
+        </is>
+      </c>
+      <c r="H948" t="inlineStr">
+        <is>
+          <t>PercentOfBase</t>
+        </is>
+      </c>
+      <c r="I948" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J948" t="n">
+        <v>213055</v>
+      </c>
+      <c r="K948" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L948" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M948" t="n">
+        <v>0</v>
+      </c>
+      <c r="P948" t="inlineStr">
+        <is>
+          <t>PercentOfBase</t>
+        </is>
+      </c>
+      <c r="Q948" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R948" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="B949" t="n">
+        <v>211056</v>
+      </c>
+      <c r="C949" t="n">
+        <v>210011</v>
+      </c>
+      <c r="E949" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F949" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G949" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H949" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I949" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J949" t="n">
+        <v>213056</v>
+      </c>
+      <c r="K949" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L949" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M949" t="n">
+        <v>0</v>
+      </c>
+      <c r="P949" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q949" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R949" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="B950" t="n">
+        <v>211057</v>
+      </c>
+      <c r="C950" t="n">
+        <v>210011</v>
+      </c>
+      <c r="E950" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F950" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G950" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H950" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I950" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J950" t="n">
+        <v>213057</v>
+      </c>
+      <c r="K950" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L950" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M950" t="n">
+        <v>0</v>
+      </c>
+      <c r="P950" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q950" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R950" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="B951" t="n">
+        <v>211058</v>
+      </c>
+      <c r="C951" t="n">
+        <v>210011</v>
+      </c>
+      <c r="E951" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F951" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G951" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H951" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I951" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J951" t="n">
+        <v>213058</v>
+      </c>
+      <c r="K951" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L951" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M951" t="n">
+        <v>0</v>
+      </c>
+      <c r="P951" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q951" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R951" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="B952" t="n">
+        <v>211059</v>
+      </c>
+      <c r="C952" t="n">
+        <v>210011</v>
+      </c>
+      <c r="E952" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F952" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G952" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H952" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I952" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J952" t="n">
+        <v>213059</v>
+      </c>
+      <c r="K952" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L952" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M952" t="n">
+        <v>0</v>
+      </c>
+      <c r="P952" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q952" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R952" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="B953" t="n">
+        <v>211060</v>
+      </c>
+      <c r="C953" t="n">
+        <v>210011</v>
+      </c>
+      <c r="E953" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F953" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G953" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H953" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I953" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J953" t="n">
+        <v>213060</v>
+      </c>
+      <c r="K953" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L953" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M953" t="n">
+        <v>0</v>
+      </c>
+      <c r="P953" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q953" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R953" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="B954" t="n">
+        <v>211061</v>
+      </c>
+      <c r="C954" t="n">
+        <v>210013</v>
+      </c>
+      <c r="E954" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F954" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G954" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H954" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I954" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J954" t="n">
+        <v>213061</v>
+      </c>
+      <c r="K954" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L954" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M954" t="n">
+        <v>0</v>
+      </c>
+      <c r="P954" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q954" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R954" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="B955" t="n">
+        <v>211062</v>
+      </c>
+      <c r="C955" t="n">
+        <v>210013</v>
+      </c>
+      <c r="E955" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F955" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G955" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H955" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I955" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J955" t="n">
+        <v>213062</v>
+      </c>
+      <c r="K955" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L955" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M955" t="n">
+        <v>0</v>
+      </c>
+      <c r="P955" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q955" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R955" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="B956" t="n">
+        <v>211063</v>
+      </c>
+      <c r="C956" t="n">
+        <v>210013</v>
+      </c>
+      <c r="E956" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F956" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G956" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H956" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I956" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J956" t="n">
+        <v>213063</v>
+      </c>
+      <c r="K956" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L956" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M956" t="n">
+        <v>0</v>
+      </c>
+      <c r="P956" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q956" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R956" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="B957" t="n">
+        <v>211064</v>
+      </c>
+      <c r="C957" t="n">
+        <v>210013</v>
+      </c>
+      <c r="E957" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F957" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G957" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H957" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I957" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J957" t="n">
+        <v>213064</v>
+      </c>
+      <c r="K957" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L957" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M957" t="n">
+        <v>0</v>
+      </c>
+      <c r="P957" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q957" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R957" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="B958" t="n">
+        <v>211065</v>
+      </c>
+      <c r="C958" t="n">
+        <v>210013</v>
+      </c>
+      <c r="E958" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F958" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G958" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H958" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I958" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J958" t="n">
+        <v>213065</v>
+      </c>
+      <c r="K958" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L958" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M958" t="n">
+        <v>0</v>
+      </c>
+      <c r="P958" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q958" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R958" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="B959" t="n">
+        <v>211066</v>
+      </c>
+      <c r="C959" t="n">
+        <v>210014</v>
+      </c>
+      <c r="E959" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F959" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G959" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H959" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I959" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J959" t="n">
+        <v>213066</v>
+      </c>
+      <c r="K959" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L959" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M959" t="n">
+        <v>0</v>
+      </c>
+      <c r="P959" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q959" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R959" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="B960" t="n">
+        <v>211067</v>
+      </c>
+      <c r="C960" t="n">
+        <v>210014</v>
+      </c>
+      <c r="E960" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F960" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G960" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H960" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I960" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J960" t="n">
+        <v>213067</v>
+      </c>
+      <c r="K960" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L960" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M960" t="n">
+        <v>0</v>
+      </c>
+      <c r="P960" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q960" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R960" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="B961" t="n">
+        <v>211068</v>
+      </c>
+      <c r="C961" t="n">
+        <v>210014</v>
+      </c>
+      <c r="E961" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F961" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G961" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H961" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I961" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J961" t="n">
+        <v>213068</v>
+      </c>
+      <c r="K961" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L961" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M961" t="n">
+        <v>0</v>
+      </c>
+      <c r="P961" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q961" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R961" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="B962" t="n">
+        <v>211069</v>
+      </c>
+      <c r="C962" t="n">
+        <v>210014</v>
+      </c>
+      <c r="E962" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F962" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G962" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H962" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I962" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J962" t="n">
+        <v>213069</v>
+      </c>
+      <c r="K962" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L962" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M962" t="n">
+        <v>0</v>
+      </c>
+      <c r="P962" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q962" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R962" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="B963" t="n">
+        <v>211070</v>
+      </c>
+      <c r="C963" t="n">
+        <v>210014</v>
+      </c>
+      <c r="E963" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F963" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G963" t="inlineStr">
+        <is>
+          <t>CritDamage</t>
+        </is>
+      </c>
+      <c r="H963" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I963" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J963" t="n">
+        <v>213070</v>
+      </c>
+      <c r="K963" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L963" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M963" t="n">
+        <v>0</v>
+      </c>
+      <c r="P963" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q963" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R963" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="B964" t="n">
+        <v>211071</v>
+      </c>
+      <c r="C964" t="n">
+        <v>210015</v>
+      </c>
+      <c r="E964" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F964" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G964" t="inlineStr">
+        <is>
+          <t>EffectHitRate</t>
+        </is>
+      </c>
+      <c r="H964" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I964" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J964" t="n">
+        <v>213071</v>
+      </c>
+      <c r="K964" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L964" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M964" t="n">
+        <v>0</v>
+      </c>
+      <c r="P964" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q964" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R964" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="B965" t="n">
+        <v>211072</v>
+      </c>
+      <c r="C965" t="n">
+        <v>210015</v>
+      </c>
+      <c r="E965" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F965" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G965" t="inlineStr">
+        <is>
+          <t>EffectHitRate</t>
+        </is>
+      </c>
+      <c r="H965" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I965" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J965" t="n">
+        <v>213072</v>
+      </c>
+      <c r="K965" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L965" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M965" t="n">
+        <v>0</v>
+      </c>
+      <c r="P965" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q965" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R965" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="B966" t="n">
+        <v>211073</v>
+      </c>
+      <c r="C966" t="n">
+        <v>210015</v>
+      </c>
+      <c r="E966" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F966" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G966" t="inlineStr">
+        <is>
+          <t>EffectHitRate</t>
+        </is>
+      </c>
+      <c r="H966" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I966" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J966" t="n">
+        <v>213073</v>
+      </c>
+      <c r="K966" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L966" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M966" t="n">
+        <v>0</v>
+      </c>
+      <c r="P966" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q966" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R966" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="B967" t="n">
+        <v>211074</v>
+      </c>
+      <c r="C967" t="n">
+        <v>210015</v>
+      </c>
+      <c r="E967" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F967" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G967" t="inlineStr">
+        <is>
+          <t>EffectHitRate</t>
+        </is>
+      </c>
+      <c r="H967" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I967" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J967" t="n">
+        <v>213074</v>
+      </c>
+      <c r="K967" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L967" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M967" t="n">
+        <v>0</v>
+      </c>
+      <c r="P967" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q967" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R967" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="B968" t="n">
+        <v>211075</v>
+      </c>
+      <c r="C968" t="n">
+        <v>210015</v>
+      </c>
+      <c r="E968" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F968" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G968" t="inlineStr">
+        <is>
+          <t>EffectHitRate</t>
+        </is>
+      </c>
+      <c r="H968" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I968" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J968" t="n">
+        <v>213075</v>
+      </c>
+      <c r="K968" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L968" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M968" t="n">
+        <v>0</v>
+      </c>
+      <c r="P968" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q968" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R968" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="B969" t="n">
+        <v>211076</v>
+      </c>
+      <c r="C969" t="n">
+        <v>210016</v>
+      </c>
+      <c r="E969" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F969" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G969" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H969" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I969" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J969" t="n">
+        <v>213076</v>
+      </c>
+      <c r="K969" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L969" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M969" t="n">
+        <v>0</v>
+      </c>
+      <c r="P969" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q969" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R969" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="B970" t="n">
+        <v>211077</v>
+      </c>
+      <c r="C970" t="n">
+        <v>210016</v>
+      </c>
+      <c r="E970" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F970" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G970" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H970" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I970" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J970" t="n">
+        <v>213077</v>
+      </c>
+      <c r="K970" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L970" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M970" t="n">
+        <v>0</v>
+      </c>
+      <c r="P970" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q970" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R970" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="B971" t="n">
+        <v>211078</v>
+      </c>
+      <c r="C971" t="n">
+        <v>210016</v>
+      </c>
+      <c r="E971" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F971" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G971" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H971" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I971" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J971" t="n">
+        <v>213078</v>
+      </c>
+      <c r="K971" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L971" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M971" t="n">
+        <v>0</v>
+      </c>
+      <c r="P971" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q971" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R971" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="B972" t="n">
+        <v>211079</v>
+      </c>
+      <c r="C972" t="n">
+        <v>210016</v>
+      </c>
+      <c r="E972" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F972" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G972" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H972" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I972" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J972" t="n">
+        <v>213079</v>
+      </c>
+      <c r="K972" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L972" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M972" t="n">
+        <v>0</v>
+      </c>
+      <c r="P972" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q972" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R972" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="B973" t="n">
+        <v>211080</v>
+      </c>
+      <c r="C973" t="n">
+        <v>210016</v>
+      </c>
+      <c r="E973" t="n">
+        <v>216001</v>
+      </c>
+      <c r="F973" t="n">
+        <v>216002</v>
+      </c>
+      <c r="G973" t="inlineStr">
+        <is>
+          <t>CritRate</t>
+        </is>
+      </c>
+      <c r="H973" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="I973" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="J973" t="n">
+        <v>213080</v>
+      </c>
+      <c r="K973" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="L973" t="n">
+        <v>216003</v>
+      </c>
+      <c r="M973" t="n">
+        <v>0</v>
+      </c>
+      <c r="P973" t="inlineStr">
+        <is>
+          <t>BaseAdd</t>
+        </is>
+      </c>
+      <c r="Q973" t="inlineStr">
+        <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="R973" t="inlineStr">
+        <is>
+          <t>Battle</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>